<commit_message>
Adopt canonical 13-column comment resolution matrix contract from spectrum-systems; require numbered PDF input
Co-authored-by: nicklasorte <37697540+nicklasorte@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/examples/comment_matrix_sample.xlsx
+++ b/outputs/examples/comment_matrix_sample.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Comment Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Comment Resolution Matrix" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,19 +454,19 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>Comment Type: Editorial/Grammar, Clarification, Technical</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>Agency Notes</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Agency Suggested Text Change</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>WG Chain Comments</t>
-        </is>
-      </c>
       <c r="K1" t="inlineStr">
         <is>
           <t>NTIA Comments</t>
@@ -480,101 +480,6 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>Resolution</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Report Context</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Resolution Task</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Comment Cluster Id</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Intent Classification</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Section Group</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>Heat Level</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>Validation Status</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>Validation Notes</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>Resolved Against Revision</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>Generation Mode</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>Rule Id</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>Rule Source</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>Rule Version</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>Rules Profile</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>Rules Profile Version</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>Matched Rule Types</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>Review Status</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>Confidence Score</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>Provenance Record Id</t>
         </is>
       </c>
     </row>
@@ -594,7 +499,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DRAFT</t>
+          <t>DRAFT-1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -614,18 +519,22 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>Technical</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>Clarify the propagation model assumptions in Section 2.3; current text implies free-space losses only.</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Specify whether clutter and diffraction losses are included in the link budget.</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Anchored to p.5 para 2: the working paper cites path loss without environment class.</t>
+          <t>Anchored to p.5 lines 14-18: the working paper cites path loss without environment class.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -636,75 +545,6 @@
       <c r="M2" t="inlineStr">
         <is>
           <t>Update Section 2.3 to include environmental loss factors and cite reference model.</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Path loss modeled as 20log10(d) with no additional factors.</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>major</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>NOT_VALIDATED</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>DRAFT</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>comment-matrix</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>rule-placeholder</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>working-paper-review-engine</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>0.0.0</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>0.0.0</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>PROPOSED</t>
-        </is>
-      </c>
-      <c r="AE2" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>comment-1</t>
         </is>
       </c>
     </row>

</xml_diff>